<commit_message>
Day 13-14 - Completed Financial Ratio Engine and Sprint Review
</commit_message>
<xml_diff>
--- a/data/raw/analysis.xlsx
+++ b/data/raw/analysis.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Narendra\Desktop\nifty100_project\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F46738F0-D05A-4B92-BCD6-9D1B44CEFF27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6B657AB-1434-4011-B0D4-4AEBCEEE78E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2304" yWindow="2304" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2964" yWindow="2964" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Analysis" sheetId="1" r:id="rId1"/>
@@ -739,7 +739,7 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
-    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="2" max="2" width="15.88671875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="33" customWidth="1"/>
     <col min="4" max="5" width="26" customWidth="1"/>
     <col min="6" max="6" width="23" customWidth="1"/>

</xml_diff>